<commit_message>
Final Secure Setup: R-Drive, Weekly Roadmap, and Fixes
</commit_message>
<xml_diff>
--- a/data/Master_Tracker_Live.xlsx
+++ b/data/Master_Tracker_Live.xlsx
@@ -1510,13 +1510,25 @@
       <c r="C4" s="10">
         <v>46153.0</v>
       </c>
-      <c r="D4" s="10"/>
+      <c r="D4" s="10">
+        <f t="shared" ref="D4:D5" si="1">C4+1</f>
+        <v>46154</v>
+      </c>
       <c r="E4" s="11"/>
-      <c r="F4" s="10"/>
+      <c r="F4" s="10">
+        <f>C4+7</f>
+        <v>46160</v>
+      </c>
       <c r="G4" s="11"/>
-      <c r="H4" s="10"/>
+      <c r="H4" s="10">
+        <f t="shared" ref="H4:H5" si="2">C4+15</f>
+        <v>46168</v>
+      </c>
       <c r="I4" s="11"/>
-      <c r="J4" s="10"/>
+      <c r="J4" s="10">
+        <f t="shared" ref="J4:J5" si="3">C4+30</f>
+        <v>46183</v>
+      </c>
       <c r="K4" s="11"/>
       <c r="L4" s="10"/>
       <c r="M4" s="11"/>
@@ -1530,13 +1542,25 @@
         <v>18</v>
       </c>
       <c r="C5" s="10"/>
-      <c r="D5" s="10"/>
+      <c r="D5" s="10">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
       <c r="E5" s="11"/>
-      <c r="F5" s="10"/>
+      <c r="F5" s="10">
+        <f>C4+1</f>
+        <v>46154</v>
+      </c>
       <c r="G5" s="11"/>
-      <c r="H5" s="10"/>
+      <c r="H5" s="10">
+        <f t="shared" si="2"/>
+        <v>15</v>
+      </c>
       <c r="I5" s="11"/>
-      <c r="J5" s="10"/>
+      <c r="J5" s="10">
+        <f t="shared" si="3"/>
+        <v>30</v>
+      </c>
       <c r="K5" s="11"/>
       <c r="L5" s="10"/>
       <c r="M5" s="11"/>
@@ -1554,7 +1578,10 @@
       <c r="E6" s="11"/>
       <c r="F6" s="10"/>
       <c r="G6" s="11"/>
-      <c r="H6" s="10"/>
+      <c r="H6" s="10">
+        <f>C4+1</f>
+        <v>46154</v>
+      </c>
       <c r="I6" s="11"/>
       <c r="J6" s="10"/>
       <c r="K6" s="11"/>
@@ -1576,7 +1603,10 @@
       <c r="G7" s="11"/>
       <c r="H7" s="10"/>
       <c r="I7" s="11"/>
-      <c r="J7" s="10"/>
+      <c r="J7" s="10">
+        <f>C4+1</f>
+        <v>46154</v>
+      </c>
       <c r="K7" s="11"/>
       <c r="L7" s="10"/>
       <c r="M7" s="11"/>
@@ -1598,7 +1628,10 @@
       <c r="I8" s="11"/>
       <c r="J8" s="10"/>
       <c r="K8" s="11"/>
-      <c r="L8" s="10"/>
+      <c r="L8" s="10">
+        <f>C4+1</f>
+        <v>46154</v>
+      </c>
       <c r="M8" s="11"/>
       <c r="N8" s="12"/>
     </row>

</xml_diff>